<commit_message>
feat(isobutanol): repoint k_16ia/k_16ie to k_17ia/k_17ie, add Adh6 (r17) rows to the six Ehrlich workbooks
nskinetics 2026-09-15 split the lumped Ehrlich step r16 (Aro10 + Adh6) into
r16 (Aro10, pure decarboxylase) + r17 (Adh6, NADPH aldehyde reductase, a
structural mirror of r6). The acetate / ethanol cross-product exponentials
moved to r17 as k_17ia / k_17ie, so the two workbook rows are repointed
(values unchanged; units fixed to l_per_g), the two Aro10 rows relabelled
Ketoisovalerate-to-Isobutyraldehyde, and four rows appended at the antimony
defaults with +-20 % bands and References transcribing the derivations:
k_17 44 g/L/h, K_17 0.0086 g/L, k_17r 2.5e-4, K_17e 0.020. B (and each
opt_*) kinetic set 55 -> 59. A untouched (k_17 inert while k_16 = 0).
build_opt_scenario_workbooks.py copies B, so its docstring only notes it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_B.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_B.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="40.81640625" customWidth="1" min="1" max="1"/>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Ketoisovalerate-to-Isobutanol</t>
+          <t>Kinetics: Ketoisovalerate-to-Isobutyraldehyde</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Ketoisovalerate-to-Isobutanol</t>
+          <t>Kinetics: Ketoisovalerate-to-Isobutyraldehyde</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>K_16 = 0.27 g/L: Aro10 (the rate-limiting decarboxylase of the lumped KDC + ADH step r16) KIV affinity, Km 8.5 mM (Kneen et al. 2011 FEBS J. 278:1842; BRENDA EC 4.1.1.43), anchored by ratio to r3's Pdc (Km 1.1 mM) exactly as K_13 was, with the molar-mass correction: (8.5/1.1) x 0.302 mM x 116.12 g/mol. r16 is irreversible Michaelis-Menten in KIV since 2026-09-13 (nskinetics b61360e; was 0.034, copied from K_6). +-20% kinetic convention (band 0.27-0.60 for Pdc Km 1.1-0.5 mM is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13).</t>
+          <t>K_16 = 0.27 g/L: Aro10 (the rate-limiting decarboxylase of the lumped KDC + ADH step r16) KIV affinity, Km 8.5 mM (Kneen et al. 2011 FEBS J. 278:1842; BRENDA EC 4.1.1.43), anchored by ratio to r3's Pdc (Km 1.1 mM) exactly as K_13 was, with the molar-mass correction: (8.5/1.1) x 0.302 mM x 116.12 g/mol. r16 is irreversible Michaelis-Menten in KIV since 2026-09-13 (nskinetics b61360e; was 0.034, copied from K_6). +-20% kinetic convention (band 0.27-0.60 for Pdc Km 1.1-0.5 mM is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13). Since the 2026-09-15 nskinetics split of the lumped step, r16 is the Aro10 decarboxylation alone (KIV -&gt; isobutyraldehyde + CO2); the Adh6 aldehyde reduction is r17 (k_17, K_17, k_17r, K_17e, k_17ia, k_17ie).</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
@@ -3781,12 +3781,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>._k_16ia</t>
+          <t>._k_17ia</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Kinetics: Ketoisovalerate-to-Isobutanol</t>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>l_per_g</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -3816,21 +3816,26 @@
       <c r="I74" t="n">
         <v>0.07199999999999999</v>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>k_17ia (L/g): acetate cross-product exponential exp(-k_17ia*s_acetate) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ia). The old k_16ia is declared inert (0) in the antimony.</t>
+        </is>
+      </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_16ia = x</t>
+          <t>V406.nsk_kinetic_model._te.k_17ia = x</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>._k_16ie</t>
+          <t>._k_17ie</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Kinetics: Ketoisovalerate-to-Isobutanol</t>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3840,7 +3845,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>l_per_g</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -3860,9 +3865,210 @@
       <c r="I75" t="n">
         <v>0.024</v>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>k_17ie (L/g): ethanol cross-product exponential exp(-k_17ie*s_EtOH) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ie). The old k_16ie is declared inert (0) in the antimony.</t>
+        </is>
+      </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_16ie = x</t>
+          <t>V406.nsk_kinetic_model._te.k_17ie = x</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>._k_17</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>g_per_l_per_h</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>44</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="H76" t="n">
+        <v>44</v>
+      </c>
+      <c r="I76" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>k_17 = 44 g/L/h: Adh6 (NADPH-dependent aldehyde reductase) capacity for the isobutyraldehyde -&gt; isobutanol step r17 of the 2026-09-15 nskinetics split of the lumped KDC + ADH step. A vmax grounded on the Adh6:Aro10 kcat ratio 296/19 (Adh6 296 s^-1 on 2-methylpropanal + NADPH, Larroy et al. 2002 Biochem. J. 361:163; Aro10 19 s^-1 on KIV, Kneen et al. 2011 FEBS J. 278:1842) x k_16's scenario-B value 2.82 g/L/h. CONSTITUTIVE (not a scenario toggle: the antimony default is 44 in every scenario, incl. A, where it is inert while k_16 = 0), set to keep Adh6 non-limiting at scenario-B flux. +-20 % kinetic convention.</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_17 = x</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>K_17</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>g_per_l</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>0.0086</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0.006880000000000001</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.0086</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.01032</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>K_17 = 0.0086 g/L: Adh6 isobutyraldehyde affinity, K_6 x (0.17/1.1) x (72.11/44.05) -- the Adh6:Adh1 aldehyde-affinity ratio (Adh6 branched-aldehyde Km 0.13-0.21 mM, midpoint 0.17 mM, Larroy et al. 2002 Biochem. J. 361:163; Adh1 acetaldehyde Km 1.1 mM, Ganzhorn et al. 1987 JBC 262:3754) applied to r6's fitted K_6 with the molar-mass correction (isobutyraldehyde 72.11 vs acetaldehyde 44.05 g/mol). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.K_17 = x</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>k_17r</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>k_17r = 2.5e-4 (dimensionless): the r17 reverse-balance ratio, k_6r/50 -- r6's fitted Adh1 reverse balance scaled by Adh6's ~50-fold aldehyde-over-alcohol preference (Larroy et al. 2002 Biochem. J. 361:163). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_17r = x</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>K_17e</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Kinetics: Isobutyraldehyde-to-Isobutanol</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>K_17e = 0.020 (dimensionless): competitive isobutanol product term of r17, K_17 / Ki_IBO,model with Ki_IBO,model = 0.70 x 50 x 0.17 mM = 0.44 g/L isobutanol (the 0.70 is r6's own in-vitro -&gt; in-vivo transfer factor read off K_6/K_6e; 50 = Adh6's aldehyde-over-alcohol preference, Larroy et al. 2002). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.K_17e = x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(isobutanol): feedstock starch content uniform 0.684-0.743 (B + opt_* workbooks)
The 'Feedstock starch content' row of the B and five opt_* parameter-
distribution workbooks goes from Triangular 0.576 / 0.72 / 0.864 to
Uniform 0.684-0.743 kg/dry-kg with a blank Midpoint (biosteam's
parameters_from_df rejects a Uniform row with a midpoint). Baseline
0.72 is unchanged. Bounds = min / max of the 2022-2024 U.S. corn starch
content (dry basis), U.S. Grains Council 2024/2025 Corn Harvest Quality
Report (https://grains.org/corn_report/corn-harvest-quality-report-2024-2025-2/),
recorded in the row's References column.

The scenario-A workbook is not included (open in Excel at the time).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_B.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_B.xlsx
@@ -1185,19 +1185,21 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Triangular</t>
+          <t>Uniform</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.576</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n">
-        <v>0.864</v>
-      </c>
-      <c r="J16" s="3" t="n"/>
+        <v>0.743</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Uniform over the min-max of the 2022-2024 U.S. corn starch content (dry basis) 68.4-74.3 %, U.S. Grains Council, 2024/2025 Corn Harvest Quality Report, https://grains.org/corn_report/corn-harvest-quality-report-2024-2025-2/</t>
+        </is>
+      </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
           <t>fixed_F_mass = feedstock.F_mass; feedstock.imass['Starch'] = x * (fixed_F_mass - feedstock.imass['Water']); feedstock.F_mass = fixed_F_mass</t>

</xml_diff>